<commit_message>
pre work files and structure
</commit_message>
<xml_diff>
--- a/pre-week-2/Homework 1 Pre-week 2.xlsx
+++ b/pre-week-2/Homework 1 Pre-week 2.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\patri\Documents\DataAnalytics-2026\pre-week-2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9999450E-9C46-46A2-A1E3-6016C1576041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAA2F1CA-F54A-447B-B988-EB384040FBF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3540" yWindow="2880" windowWidth="28800" windowHeight="15345" xr2:uid="{751EEC58-CE82-47CC-8A34-FB2CB968C717}"/>
+    <workbookView xWindow="-26370" yWindow="7650" windowWidth="21045" windowHeight="13290" xr2:uid="{751EEC58-CE82-47CC-8A34-FB2CB968C717}"/>
   </bookViews>
   <sheets>
     <sheet name="HW 1" sheetId="2" r:id="rId1"/>
-    <sheet name="HW 2" sheetId="1" r:id="rId2"/>
+    <sheet name="Store_Data" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -537,576 +537,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>'HW 2'!$A$2:$A$13</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>Store A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Store B</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Store C</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Store D</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Store E</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Store F</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Store G</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Store H</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Store I</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Store J</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Store K</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Store L</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'HW 2'!$B$2:$B$13</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>51</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>44</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>49</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>46</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>52</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>47</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>45</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>72</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>43</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>48</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>46</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>50</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-08DC-4E03-BF3C-A74F99C46793}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>'HW 2'!$A$2:$A$13</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>Store A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Store B</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Store C</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Store D</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Store E</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Store F</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Store G</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Store H</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Store I</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Store J</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Store K</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Store L</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'HW 2'!$C$2:$C$13</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-08DC-4E03-BF3C-A74F99C46793}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent3"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>'HW 2'!$A$2:$A$13</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>Store A</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Store B</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Store C</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Store D</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Store E</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Store F</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Store G</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Store H</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Store I</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Store J</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Store K</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Store L</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'HW 2'!$D$2:$D$13</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>49.416666666666664</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>47.5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>46</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>29</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>7.6331613054586773</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2.9076701075853588</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-08DC-4E03-BF3C-A74F99C46793}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
-        <c:axId val="777426632"/>
-        <c:axId val="777420872"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="777426632"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="777420872"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="777420872"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="777426632"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1649,509 +1080,6 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -2173,47 +1101,6 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C857D38-475C-E8BA-BD18-8D79CDA80AC7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>52387</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>371475</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>128587</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C371381-43FF-FF08-A5EE-540BC9439CD7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2884,6 +1771,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>